<commit_message>
Refactor migrated blocks into base-block variants
The home-page migration created fork block folders; refactor them into
option-class variants on the existing base blocks (the idiomatic EDS pattern):

- carousel-hero  -> blocks/carousel + `hero-img` option (carousel did not
  exist in the repo, so a base carousel block is added)
- columns-featured -> columns `featured` option
- cards-article    -> cards `article` option
- hero-banner      -> hero `banner` option

Variant styling folded into the base blocks' CSS, scoped to the option class
(.cards.article, .columns.featured, .hero.banner, .carousel.hero-img). Fork
folders deleted. Parsers emit `Name (variant)` via createBlock variants;
page-templates.json + import script updated to base names; content re-imported.

Notes: renamed the carousel option to `hero-img` to avoid colliding with the
existing `hero` block's CSS; set base carousel img height:auto so the variant
aspect-ratio/height drives slide sizing.
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-home.report.xlsx
+++ b/tools/importer/reports/import-home.report.xlsx
@@ -40,7 +40,7 @@
     <t>us/en.report.json</t>
   </si>
   <si>
-    <t>["carousel-hero","columns-featured","cards-article","cards-article","hero-banner","hero-banner","hero-banner","hero-banner"]</t>
+    <t>["carousel","columns","cards","cards","hero","hero","hero","hero"]</t>
   </si>
   <si>
     <t>us/en</t>
@@ -52,7 +52,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-09-12T18:19:28.780Z</t>
+    <t>2026-09-13T12:31:46.320Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>

</xml_diff>